<commit_message>
data: add draw 1237
</commit_message>
<xml_diff>
--- a/로또 회차별 당첨번호.xlsx
+++ b/로또 회차별 당첨번호.xlsx
@@ -568,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1237"/>
+  <dimension ref="A1:L1238"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="17.4"/>
   <cols>
     <col width="7.69921875" bestFit="1" customWidth="1" style="11" min="1" max="1"/>
@@ -54963,29 +54963,55 @@
       </c>
     </row>
     <row r="1237">
-      <c r="B1237" t="n">
+      <c r="B1237" s="0" t="n">
         <v>1236</v>
       </c>
-      <c r="C1237" t="n">
+      <c r="C1237" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="D1237" t="n">
+      <c r="D1237" s="0" t="n">
         <v>18</v>
       </c>
-      <c r="E1237" t="n">
+      <c r="E1237" s="0" t="n">
         <v>21</v>
       </c>
-      <c r="F1237" t="n">
+      <c r="F1237" s="0" t="n">
         <v>29</v>
       </c>
-      <c r="G1237" t="n">
+      <c r="G1237" s="0" t="n">
         <v>34</v>
       </c>
-      <c r="H1237" t="n">
+      <c r="H1237" s="0" t="n">
         <v>38</v>
       </c>
-      <c r="I1237" t="n">
+      <c r="I1237" s="0" t="n">
         <v>10</v>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="B1238" t="n">
+        <v>1237</v>
+      </c>
+      <c r="C1238" t="n">
+        <v>10</v>
+      </c>
+      <c r="D1238" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1238" t="n">
+        <v>23</v>
+      </c>
+      <c r="F1238" t="n">
+        <v>34</v>
+      </c>
+      <c r="G1238" t="n">
+        <v>37</v>
+      </c>
+      <c r="H1238" t="n">
+        <v>40</v>
+      </c>
+      <c r="I1238" t="n">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: add draw 1238
</commit_message>
<xml_diff>
--- a/로또 회차별 당첨번호.xlsx
+++ b/로또 회차별 당첨번호.xlsx
@@ -568,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1238"/>
+  <dimension ref="A1:L1239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="17.4"/>
   <cols>
     <col width="7.69921875" bestFit="1" customWidth="1" style="11" min="1" max="1"/>
@@ -54989,29 +54989,55 @@
       </c>
     </row>
     <row r="1238">
-      <c r="B1238" t="n">
+      <c r="B1238" s="0" t="n">
         <v>1237</v>
       </c>
-      <c r="C1238" t="n">
+      <c r="C1238" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="D1238" t="n">
+      <c r="D1238" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="E1238" t="n">
+      <c r="E1238" s="0" t="n">
         <v>23</v>
       </c>
-      <c r="F1238" t="n">
+      <c r="F1238" s="0" t="n">
         <v>34</v>
       </c>
-      <c r="G1238" t="n">
+      <c r="G1238" s="0" t="n">
         <v>37</v>
       </c>
-      <c r="H1238" t="n">
+      <c r="H1238" s="0" t="n">
         <v>40</v>
       </c>
-      <c r="I1238" t="n">
+      <c r="I1238" s="0" t="n">
         <v>39</v>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="B1239" t="n">
+        <v>1238</v>
+      </c>
+      <c r="C1239" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1239" t="n">
+        <v>13</v>
+      </c>
+      <c r="E1239" t="n">
+        <v>18</v>
+      </c>
+      <c r="F1239" t="n">
+        <v>32</v>
+      </c>
+      <c r="G1239" t="n">
+        <v>38</v>
+      </c>
+      <c r="H1239" t="n">
+        <v>42</v>
+      </c>
+      <c r="I1239" t="n">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: add draw 1239
</commit_message>
<xml_diff>
--- a/로또 회차별 당첨번호.xlsx
+++ b/로또 회차별 당첨번호.xlsx
@@ -568,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1239"/>
+  <dimension ref="A1:L1240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="17.4"/>
   <cols>
     <col width="7.69921875" bestFit="1" customWidth="1" style="11" min="1" max="1"/>
@@ -55015,29 +55015,55 @@
       </c>
     </row>
     <row r="1239">
-      <c r="B1239" t="n">
+      <c r="B1239" s="0" t="n">
         <v>1238</v>
       </c>
-      <c r="C1239" t="n">
+      <c r="C1239" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="D1239" t="n">
+      <c r="D1239" s="0" t="n">
         <v>13</v>
       </c>
-      <c r="E1239" t="n">
+      <c r="E1239" s="0" t="n">
         <v>18</v>
       </c>
-      <c r="F1239" t="n">
+      <c r="F1239" s="0" t="n">
         <v>32</v>
       </c>
-      <c r="G1239" t="n">
+      <c r="G1239" s="0" t="n">
         <v>38</v>
       </c>
-      <c r="H1239" t="n">
+      <c r="H1239" s="0" t="n">
         <v>42</v>
       </c>
-      <c r="I1239" t="n">
+      <c r="I1239" s="0" t="n">
         <v>22</v>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="B1240" t="n">
+        <v>1239</v>
+      </c>
+      <c r="C1240" t="n">
+        <v>11</v>
+      </c>
+      <c r="D1240" t="n">
+        <v>13</v>
+      </c>
+      <c r="E1240" t="n">
+        <v>22</v>
+      </c>
+      <c r="F1240" t="n">
+        <v>32</v>
+      </c>
+      <c r="G1240" t="n">
+        <v>33</v>
+      </c>
+      <c r="H1240" t="n">
+        <v>36</v>
+      </c>
+      <c r="I1240" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: add draw 1240
</commit_message>
<xml_diff>
--- a/로또 회차별 당첨번호.xlsx
+++ b/로또 회차별 당첨번호.xlsx
@@ -568,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1240"/>
+  <dimension ref="A1:L1241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="17.4"/>
   <cols>
     <col width="7.69921875" bestFit="1" customWidth="1" style="11" min="1" max="1"/>
@@ -55041,29 +55041,55 @@
       </c>
     </row>
     <row r="1240">
-      <c r="B1240" t="n">
+      <c r="B1240" s="0" t="n">
         <v>1239</v>
       </c>
-      <c r="C1240" t="n">
+      <c r="C1240" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="D1240" t="n">
+      <c r="D1240" s="0" t="n">
         <v>13</v>
       </c>
-      <c r="E1240" t="n">
+      <c r="E1240" s="0" t="n">
         <v>22</v>
       </c>
-      <c r="F1240" t="n">
+      <c r="F1240" s="0" t="n">
         <v>32</v>
       </c>
-      <c r="G1240" t="n">
+      <c r="G1240" s="0" t="n">
         <v>33</v>
       </c>
-      <c r="H1240" t="n">
+      <c r="H1240" s="0" t="n">
         <v>36</v>
       </c>
-      <c r="I1240" t="n">
+      <c r="I1240" s="0" t="n">
         <v>8</v>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="B1241" t="n">
+        <v>1240</v>
+      </c>
+      <c r="C1241" t="n">
+        <v>11</v>
+      </c>
+      <c r="D1241" t="n">
+        <v>13</v>
+      </c>
+      <c r="E1241" t="n">
+        <v>19</v>
+      </c>
+      <c r="F1241" t="n">
+        <v>20</v>
+      </c>
+      <c r="G1241" t="n">
+        <v>31</v>
+      </c>
+      <c r="H1241" t="n">
+        <v>44</v>
+      </c>
+      <c r="I1241" t="n">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: add draw 1241
</commit_message>
<xml_diff>
--- a/로또 회차별 당첨번호.xlsx
+++ b/로또 회차별 당첨번호.xlsx
@@ -568,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1241"/>
+  <dimension ref="A1:L1242"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="17.4"/>
   <cols>
     <col width="7.69921875" bestFit="1" customWidth="1" style="11" min="1" max="1"/>
@@ -55067,29 +55067,55 @@
       </c>
     </row>
     <row r="1241">
-      <c r="B1241" t="n">
+      <c r="B1241" s="0" t="n">
         <v>1240</v>
       </c>
-      <c r="C1241" t="n">
+      <c r="C1241" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="D1241" t="n">
+      <c r="D1241" s="0" t="n">
         <v>13</v>
       </c>
-      <c r="E1241" t="n">
+      <c r="E1241" s="0" t="n">
         <v>19</v>
       </c>
-      <c r="F1241" t="n">
+      <c r="F1241" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="G1241" t="n">
+      <c r="G1241" s="0" t="n">
         <v>31</v>
       </c>
-      <c r="H1241" t="n">
+      <c r="H1241" s="0" t="n">
         <v>44</v>
       </c>
-      <c r="I1241" t="n">
+      <c r="I1241" s="0" t="n">
         <v>27</v>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="B1242" t="n">
+        <v>1241</v>
+      </c>
+      <c r="C1242" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1242" t="n">
+        <v>13</v>
+      </c>
+      <c r="E1242" t="n">
+        <v>16</v>
+      </c>
+      <c r="F1242" t="n">
+        <v>23</v>
+      </c>
+      <c r="G1242" t="n">
+        <v>24</v>
+      </c>
+      <c r="H1242" t="n">
+        <v>43</v>
+      </c>
+      <c r="I1242" t="n">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: add draw 1242
</commit_message>
<xml_diff>
--- a/로또 회차별 당첨번호.xlsx
+++ b/로또 회차별 당첨번호.xlsx
@@ -568,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1242"/>
+  <dimension ref="A1:L1243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="17.4"/>
   <cols>
     <col width="7.69921875" bestFit="1" customWidth="1" style="11" min="1" max="1"/>
@@ -55093,28 +55093,54 @@
       </c>
     </row>
     <row r="1242">
-      <c r="B1242" t="n">
+      <c r="B1242" s="0" t="n">
         <v>1241</v>
       </c>
-      <c r="C1242" t="n">
+      <c r="C1242" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="D1242" t="n">
+      <c r="D1242" s="0" t="n">
         <v>13</v>
       </c>
-      <c r="E1242" t="n">
+      <c r="E1242" s="0" t="n">
         <v>16</v>
       </c>
-      <c r="F1242" t="n">
+      <c r="F1242" s="0" t="n">
         <v>23</v>
       </c>
-      <c r="G1242" t="n">
+      <c r="G1242" s="0" t="n">
         <v>24</v>
       </c>
-      <c r="H1242" t="n">
+      <c r="H1242" s="0" t="n">
         <v>43</v>
       </c>
-      <c r="I1242" t="n">
+      <c r="I1242" s="0" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="B1243" t="n">
+        <v>1242</v>
+      </c>
+      <c r="C1243" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1243" t="n">
+        <v>4</v>
+      </c>
+      <c r="E1243" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1243" t="n">
+        <v>16</v>
+      </c>
+      <c r="G1243" t="n">
+        <v>31</v>
+      </c>
+      <c r="H1243" t="n">
+        <v>41</v>
+      </c>
+      <c r="I1243" t="n">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: add draw 1243
</commit_message>
<xml_diff>
--- a/로또 회차별 당첨번호.xlsx
+++ b/로또 회차별 당첨번호.xlsx
@@ -568,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1243"/>
+  <dimension ref="A1:L1244"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="17.4"/>
   <cols>
     <col width="7.69921875" bestFit="1" customWidth="1" style="11" min="1" max="1"/>
@@ -55119,29 +55119,55 @@
       </c>
     </row>
     <row r="1243">
-      <c r="B1243" t="n">
+      <c r="B1243" s="0" t="n">
         <v>1242</v>
       </c>
-      <c r="C1243" t="n">
+      <c r="C1243" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="D1243" t="n">
+      <c r="D1243" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="E1243" t="n">
+      <c r="E1243" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="F1243" t="n">
+      <c r="F1243" s="0" t="n">
         <v>16</v>
       </c>
-      <c r="G1243" t="n">
+      <c r="G1243" s="0" t="n">
         <v>31</v>
       </c>
-      <c r="H1243" t="n">
+      <c r="H1243" s="0" t="n">
         <v>41</v>
       </c>
-      <c r="I1243" t="n">
+      <c r="I1243" s="0" t="n">
         <v>9</v>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="B1244" t="n">
+        <v>1243</v>
+      </c>
+      <c r="C1244" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1244" t="n">
+        <v>18</v>
+      </c>
+      <c r="E1244" t="n">
+        <v>24</v>
+      </c>
+      <c r="F1244" t="n">
+        <v>38</v>
+      </c>
+      <c r="G1244" t="n">
+        <v>43</v>
+      </c>
+      <c r="H1244" t="n">
+        <v>44</v>
+      </c>
+      <c r="I1244" t="n">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: add draw 1244
</commit_message>
<xml_diff>
--- a/로또 회차별 당첨번호.xlsx
+++ b/로또 회차별 당첨번호.xlsx
@@ -568,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1244"/>
+  <dimension ref="A1:L1245"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="17.4"/>
   <cols>
     <col width="7.69921875" bestFit="1" customWidth="1" style="11" min="1" max="1"/>
@@ -55145,29 +55145,55 @@
       </c>
     </row>
     <row r="1244">
-      <c r="B1244" t="n">
+      <c r="B1244" s="0" t="n">
         <v>1243</v>
       </c>
-      <c r="C1244" t="n">
+      <c r="C1244" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="D1244" t="n">
+      <c r="D1244" s="0" t="n">
         <v>18</v>
       </c>
-      <c r="E1244" t="n">
+      <c r="E1244" s="0" t="n">
         <v>24</v>
       </c>
-      <c r="F1244" t="n">
+      <c r="F1244" s="0" t="n">
         <v>38</v>
       </c>
-      <c r="G1244" t="n">
+      <c r="G1244" s="0" t="n">
         <v>43</v>
       </c>
-      <c r="H1244" t="n">
+      <c r="H1244" s="0" t="n">
         <v>44</v>
       </c>
-      <c r="I1244" t="n">
+      <c r="I1244" s="0" t="n">
         <v>35</v>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="B1245" t="n">
+        <v>1244</v>
+      </c>
+      <c r="C1245" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1245" t="n">
+        <v>13</v>
+      </c>
+      <c r="E1245" t="n">
+        <v>18</v>
+      </c>
+      <c r="F1245" t="n">
+        <v>26</v>
+      </c>
+      <c r="G1245" t="n">
+        <v>34</v>
+      </c>
+      <c r="H1245" t="n">
+        <v>38</v>
+      </c>
+      <c r="I1245" t="n">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: add draw 1245
</commit_message>
<xml_diff>
--- a/로또 회차별 당첨번호.xlsx
+++ b/로또 회차별 당첨번호.xlsx
@@ -568,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1245"/>
+  <dimension ref="A1:L1246"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="17.4"/>
   <cols>
     <col width="7.69921875" bestFit="1" customWidth="1" style="11" min="1" max="1"/>
@@ -55171,29 +55171,55 @@
       </c>
     </row>
     <row r="1245">
-      <c r="B1245" t="n">
+      <c r="B1245" s="0" t="n">
         <v>1244</v>
       </c>
-      <c r="C1245" t="n">
+      <c r="C1245" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="D1245" t="n">
+      <c r="D1245" s="0" t="n">
         <v>13</v>
       </c>
-      <c r="E1245" t="n">
+      <c r="E1245" s="0" t="n">
         <v>18</v>
       </c>
-      <c r="F1245" t="n">
+      <c r="F1245" s="0" t="n">
         <v>26</v>
       </c>
-      <c r="G1245" t="n">
+      <c r="G1245" s="0" t="n">
         <v>34</v>
       </c>
-      <c r="H1245" t="n">
+      <c r="H1245" s="0" t="n">
         <v>38</v>
       </c>
-      <c r="I1245" t="n">
+      <c r="I1245" s="0" t="n">
         <v>25</v>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="B1246" t="n">
+        <v>1245</v>
+      </c>
+      <c r="C1246" t="n">
+        <v>4</v>
+      </c>
+      <c r="D1246" t="n">
+        <v>5</v>
+      </c>
+      <c r="E1246" t="n">
+        <v>25</v>
+      </c>
+      <c r="F1246" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1246" t="n">
+        <v>32</v>
+      </c>
+      <c r="H1246" t="n">
+        <v>42</v>
+      </c>
+      <c r="I1246" t="n">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: add draw 1246
</commit_message>
<xml_diff>
--- a/로또 회차별 당첨번호.xlsx
+++ b/로또 회차별 당첨번호.xlsx
@@ -568,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1246"/>
+  <dimension ref="A1:L1247"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="17.4"/>
   <cols>
     <col width="7.69921875" bestFit="1" customWidth="1" style="11" min="1" max="1"/>
@@ -55197,29 +55197,55 @@
       </c>
     </row>
     <row r="1246">
-      <c r="B1246" t="n">
+      <c r="B1246" s="0" t="n">
         <v>1245</v>
       </c>
-      <c r="C1246" t="n">
+      <c r="C1246" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="D1246" t="n">
+      <c r="D1246" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="E1246" t="n">
+      <c r="E1246" s="0" t="n">
         <v>25</v>
       </c>
-      <c r="F1246" t="n">
+      <c r="F1246" s="0" t="n">
         <v>28</v>
       </c>
-      <c r="G1246" t="n">
+      <c r="G1246" s="0" t="n">
         <v>32</v>
       </c>
-      <c r="H1246" t="n">
+      <c r="H1246" s="0" t="n">
         <v>42</v>
       </c>
-      <c r="I1246" t="n">
+      <c r="I1246" s="0" t="n">
         <v>12</v>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="B1247" t="n">
+        <v>1246</v>
+      </c>
+      <c r="C1247" t="n">
+        <v>16</v>
+      </c>
+      <c r="D1247" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1247" t="n">
+        <v>23</v>
+      </c>
+      <c r="F1247" t="n">
+        <v>24</v>
+      </c>
+      <c r="G1247" t="n">
+        <v>27</v>
+      </c>
+      <c r="H1247" t="n">
+        <v>28</v>
+      </c>
+      <c r="I1247" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: add draw 1247
</commit_message>
<xml_diff>
--- a/로또 회차별 당첨번호.xlsx
+++ b/로또 회차별 당첨번호.xlsx
@@ -568,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1247"/>
+  <dimension ref="A1:L1248"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="17.4"/>
   <cols>
     <col width="7.69921875" bestFit="1" customWidth="1" style="11" min="1" max="1"/>
@@ -55223,29 +55223,55 @@
       </c>
     </row>
     <row r="1247">
-      <c r="B1247" t="n">
+      <c r="B1247" s="0" t="n">
         <v>1246</v>
       </c>
-      <c r="C1247" t="n">
+      <c r="C1247" s="0" t="n">
         <v>16</v>
       </c>
-      <c r="D1247" t="n">
+      <c r="D1247" s="0" t="n">
         <v>22</v>
       </c>
-      <c r="E1247" t="n">
+      <c r="E1247" s="0" t="n">
         <v>23</v>
       </c>
-      <c r="F1247" t="n">
+      <c r="F1247" s="0" t="n">
         <v>24</v>
       </c>
-      <c r="G1247" t="n">
+      <c r="G1247" s="0" t="n">
         <v>27</v>
       </c>
-      <c r="H1247" t="n">
+      <c r="H1247" s="0" t="n">
         <v>28</v>
       </c>
-      <c r="I1247" t="n">
+      <c r="I1247" s="0" t="n">
         <v>6</v>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="B1248" t="n">
+        <v>1247</v>
+      </c>
+      <c r="C1248" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1248" t="n">
+        <v>14</v>
+      </c>
+      <c r="E1248" t="n">
+        <v>21</v>
+      </c>
+      <c r="F1248" t="n">
+        <v>22</v>
+      </c>
+      <c r="G1248" t="n">
+        <v>42</v>
+      </c>
+      <c r="H1248" t="n">
+        <v>45</v>
+      </c>
+      <c r="I1248" t="n">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>